<commit_message>
Update Excel Algoritma Raporu sheet with new logic
</commit_message>
<xml_diff>
--- a/dashboard/public/YetGen_Gruplar.xlsx
+++ b/dashboard/public/YetGen_Gruplar.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5299" uniqueCount="723">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5321" uniqueCount="701">
   <si>
     <t>Grup No</t>
   </si>
@@ -2119,10 +2119,10 @@
     <t>1. Algoritma ve Puanlama Mantığı:</t>
   </si>
   <si>
-    <t>Algoritma, katılımcıları form tercihlerine göre birbirleriyle eşleştirir. En yüksek ağırlık (20 puan) 'Önerilen Konu' ve ortak 'Hedef Kitle'lere verilmiştir. Daha sonra 1. Tercih (10p), 2. Tercih (7p) ve 3. Tercih (4p) dikkate alınarak kişilerin birbirlerine olan 'Uyum Skoru' hesaplanır. Her kişi, kendine en çok benzeyen kişilerin olduğu gruba atanır. Son olarak takas (swap) işlemi yapılarak grupların genel uyumu maksimuma çıkarılır.</t>
-  </si>
-  <si>
-    <t>2. Grup Uyum Skorları ve Detaylar:</t>
+    <t>Algoritma, oluşturulan 21 gruba baştan 7 proje konusunun her birinden 3'er tane olacak şekilde sabit profiller (Konu ve Hedef Kitle) atar. Katılımcılar gruplara dağıtılırken, kişinin önerilen konusu ile grubun atanan konusu örtüşüyorsa yüksek bonus puan alır (+30). Ayrıca kişinin tercih ettiği hedef kitle ile grubun kitle odak noktası örtüşüyorsa ek puan (+15) verilir. Kapasite kısıtlamaları dâhilinde, herkesin en uygun gruba düşmesi ve genel uyumun en yüksek seviyede tutulması sağlanır.</t>
+  </si>
+  <si>
+    <t>2. Grup Özellikleri ve Detaylar:</t>
   </si>
   <si>
     <t>Grup Adı</t>
@@ -2131,86 +2131,20 @@
     <t>Kişi Sayısı</t>
   </si>
   <si>
-    <t>Ortalama Uyum Skoru ve Açıklama</t>
-  </si>
-  <si>
-    <t>Toplam: 26 (Rastgele Atanan: 13)</t>
-  </si>
-  <si>
-    <t>Skor: 52.90  |  Yüksek Uyum (Grup üyelerinin büyük bölümü ortak konularda buluşmuş)</t>
-  </si>
-  <si>
-    <t>Skor: 82.95  |  Çok Yüksek Uyum (Grup üyelerinin hedefleri ve konuları neredeyse birebir örtüşüyor)</t>
-  </si>
-  <si>
-    <t>Skor: 69.74  |  Çok Yüksek Uyum (Grup üyelerinin hedefleri ve konuları neredeyse birebir örtüşüyor)</t>
-  </si>
-  <si>
-    <t>Skor: 48.79  |  Yüksek Uyum (Grup üyelerinin büyük bölümü ortak konularda buluşmuş)</t>
-  </si>
-  <si>
-    <t>Skor: 37.44  |  Normal Uyum (Ortak tercihleri var, ancak konular biraz daha çeşitlilik gösteriyor)</t>
-  </si>
-  <si>
-    <t>Skor: 139.37  |  Çok Yüksek Uyum (Grup üyelerinin hedefleri ve konuları neredeyse birebir örtüşüyor)</t>
-  </si>
-  <si>
-    <t>Skor: 146.33  |  Çok Yüksek Uyum (Grup üyelerinin hedefleri ve konuları neredeyse birebir örtüşüyor)</t>
-  </si>
-  <si>
-    <t>Skor: 41.55  |  Yüksek Uyum (Grup üyelerinin büyük bölümü ortak konularda buluşmuş)</t>
-  </si>
-  <si>
-    <t>Skor: 65.95  |  Çok Yüksek Uyum (Grup üyelerinin hedefleri ve konuları neredeyse birebir örtüşüyor)</t>
-  </si>
-  <si>
-    <t>Skor: 63.85  |  Çok Yüksek Uyum (Grup üyelerinin hedefleri ve konuları neredeyse birebir örtüşüyor)</t>
-  </si>
-  <si>
-    <t>Skor: 63.59  |  Çok Yüksek Uyum (Grup üyelerinin hedefleri ve konuları neredeyse birebir örtüşüyor)</t>
-  </si>
-  <si>
-    <t>Skor: 55.04  |  Yüksek Uyum (Grup üyelerinin büyük bölümü ortak konularda buluşmuş)</t>
-  </si>
-  <si>
-    <t>Toplam: 21 (Rastgele Atanan: 13)</t>
-  </si>
-  <si>
-    <t>Skor: 41.14  |  Yüksek Uyum (Grup üyelerinin büyük bölümü ortak konularda buluşmuş)</t>
-  </si>
-  <si>
-    <t>Skor: 61.78  |  Çok Yüksek Uyum (Grup üyelerinin hedefleri ve konuları neredeyse birebir örtüşüyor)</t>
-  </si>
-  <si>
-    <t>Skor: 52.10  |  Yüksek Uyum (Grup üyelerinin büyük bölümü ortak konularda buluşmuş)</t>
-  </si>
-  <si>
-    <t>Skor: 68.14  |  Çok Yüksek Uyum (Grup üyelerinin hedefleri ve konuları neredeyse birebir örtüşüyor)</t>
-  </si>
-  <si>
-    <t>Skor: 53.95  |  Yüksek Uyum (Grup üyelerinin büyük bölümü ortak konularda buluşmuş)</t>
-  </si>
-  <si>
-    <t>Skor: 50.24  |  Yüksek Uyum (Grup üyelerinin büyük bölümü ortak konularda buluşmuş)</t>
-  </si>
-  <si>
-    <t>Skor: 50.45  |  Yüksek Uyum (Grup üyelerinin büyük bölümü ortak konularda buluşmuş)</t>
-  </si>
-  <si>
-    <t>Toplam: 25 (Rastgele Atanan: 12)</t>
-  </si>
-  <si>
-    <t>Skor: 157.74  |  Çok Yüksek Uyum (Grup üyelerinin hedefleri ve konuları neredeyse birebir örtüşüyor)</t>
-  </si>
-  <si>
-    <t>Skor: 61.35  |  Çok Yüksek Uyum (Grup üyelerinin hedefleri ve konuları neredeyse birebir örtüşüyor)</t>
+    <t>26 Kişi</t>
+  </si>
+  <si>
+    <t>21 Kişi</t>
+  </si>
+  <si>
+    <t>25 Kişi</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="8">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2252,27 +2186,13 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF9C5700"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
+      <color rgb="FF334155"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2293,19 +2213,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
+        <fgColor rgb="FFF8FAFC"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2337,7 +2245,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -2352,8 +2260,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -13589,7 +13495,7 @@
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.7109375" customWidth="1"/>
@@ -13597,44 +13503,48 @@
     <col min="3" max="3" width="100.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:4">
       <c r="A1" s="2" t="s">
         <v>692</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:4">
       <c r="A3" s="3" t="s">
         <v>693</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:4">
       <c r="A4" s="4" t="s">
         <v>694</v>
       </c>
       <c r="B4" s="4"/>
       <c r="C4" s="4"/>
-    </row>
-    <row r="5" spans="1:3">
+      <c r="D4" s="4"/>
+    </row>
+    <row r="5" spans="1:4">
       <c r="A5" s="4"/>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
-    </row>
-    <row r="6" spans="1:3">
+      <c r="D5" s="4"/>
+    </row>
+    <row r="6" spans="1:4">
       <c r="A6" s="4"/>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
-    </row>
-    <row r="7" spans="1:3">
+      <c r="D6" s="4"/>
+    </row>
+    <row r="7" spans="1:4">
       <c r="A7" s="4"/>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
-    </row>
-    <row r="9" spans="1:3">
+      <c r="D7" s="4"/>
+    </row>
+    <row r="9" spans="1:4">
       <c r="A9" s="3" t="s">
         <v>695</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:4">
       <c r="A10" s="5" t="s">
         <v>696</v>
       </c>
@@ -13642,243 +13552,309 @@
         <v>697</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>698</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3">
+        <v>1</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
       <c r="A11" s="6" t="s">
         <v>9</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3">
+        <v>10</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
       <c r="A12" s="6" t="s">
         <v>50</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>699</v>
-      </c>
-      <c r="C12" s="8" t="s">
-        <v>701</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3">
+        <v>698</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
       <c r="A13" s="6" t="s">
         <v>86</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>699</v>
-      </c>
-      <c r="C13" s="8" t="s">
-        <v>702</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3">
+        <v>698</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
       <c r="A14" s="6" t="s">
         <v>124</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>703</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3">
+        <v>41</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
       <c r="A15" s="6" t="s">
         <v>153</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>699</v>
-      </c>
-      <c r="C15" s="9" t="s">
-        <v>704</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3">
+        <v>698</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
       <c r="A16" s="6" t="s">
         <v>183</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>699</v>
-      </c>
-      <c r="C16" s="8" t="s">
-        <v>705</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3">
+        <v>698</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
       <c r="A17" s="6" t="s">
         <v>220</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>699</v>
-      </c>
-      <c r="C17" s="8" t="s">
-        <v>706</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3">
+        <v>698</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
       <c r="A18" s="6" t="s">
         <v>257</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>707</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3">
+        <v>39</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
       <c r="A19" s="6" t="s">
         <v>289</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>699</v>
-      </c>
-      <c r="C19" s="8" t="s">
-        <v>708</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3">
+        <v>698</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
       <c r="A20" s="6" t="s">
         <v>322</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>699</v>
-      </c>
-      <c r="C20" s="8" t="s">
-        <v>709</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3">
+        <v>698</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
       <c r="A21" s="6" t="s">
         <v>357</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>699</v>
-      </c>
-      <c r="C21" s="8" t="s">
-        <v>710</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3">
+        <v>698</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
       <c r="A22" s="6" t="s">
         <v>394</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>711</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3">
+        <v>42</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
       <c r="A23" s="6" t="s">
         <v>423</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>712</v>
+        <v>699</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>713</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3">
+        <v>44</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4">
       <c r="A24" s="6" t="s">
         <v>446</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>699</v>
-      </c>
-      <c r="C24" s="8" t="s">
-        <v>714</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3">
+        <v>698</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
       <c r="A25" s="6" t="s">
         <v>476</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>715</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3">
+        <v>44</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
       <c r="A26" s="6" t="s">
         <v>504</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>699</v>
-      </c>
-      <c r="C26" s="8" t="s">
-        <v>716</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3">
+        <v>698</v>
+      </c>
+      <c r="C26" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
       <c r="A27" s="6" t="s">
         <v>535</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>717</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3">
+        <v>43</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
       <c r="A28" s="6" t="s">
         <v>564</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>718</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3">
+        <v>43</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4">
       <c r="A29" s="6" t="s">
         <v>597</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>719</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3">
+        <v>40</v>
+      </c>
+      <c r="D29" s="7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4">
       <c r="A30" s="6" t="s">
         <v>624</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>720</v>
-      </c>
-      <c r="C30" s="8" t="s">
-        <v>721</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3">
+        <v>700</v>
+      </c>
+      <c r="C30" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30" s="7" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4">
       <c r="A31" s="6" t="s">
         <v>659</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>720</v>
-      </c>
-      <c r="C31" s="8" t="s">
-        <v>722</v>
+        <v>700</v>
+      </c>
+      <c r="C31" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D31" s="7" t="s">
+        <v>181</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A4:C7"/>
+    <mergeCell ref="A4:D7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>